<commit_message>
Finish uncleaning and cleaning datasets. Issues log updated
</commit_message>
<xml_diff>
--- a/project/CLEAN_DATASETS/issues_log.xlsx
+++ b/project/CLEAN_DATASETS/issues_log.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vfrancisco\Desktop\repos\gacelapay_fraud_analysis\project\CLEAN_DATASETS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C96BFEF4-92F5-4272-8F7B-01BAA7C5E1F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8042A5-9142-45DC-8D49-D05C684AA335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46F2C2DC-CD36-48EA-89A3-B17E2329398E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{46F2C2DC-CD36-48EA-89A3-B17E2329398E}"/>
   </bookViews>
   <sheets>
     <sheet name="CURRENCY_EXCHANGE_RATES" sheetId="2" r:id="rId1"/>
     <sheet name="ACCOUNTS" sheetId="1" r:id="rId2"/>
     <sheet name="CUSTOMERS" sheetId="3" r:id="rId3"/>
+    <sheet name="FRAUD_DECISIONS" sheetId="4" r:id="rId4"/>
+    <sheet name="TRANSACTIONS" sheetId="5" r:id="rId5"/>
+    <sheet name="FRAUD_COSTS" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="74">
   <si>
     <t>COLUMN</t>
   </si>
@@ -229,6 +232,90 @@
   </si>
   <si>
     <t>Used REPLACE to get rid of those characters.</t>
+  </si>
+  <si>
+    <t>Not an issue, but column is unnecessary for analysis, since it maintains a 1-1 relationship the the main fact table TRANSACTIONS.</t>
+  </si>
+  <si>
+    <t>Not included in clean dataset.</t>
+  </si>
+  <si>
+    <t>ML_SCORE</t>
+  </si>
+  <si>
+    <t>Scores are coming wrapped in double quotes</t>
+  </si>
+  <si>
+    <t>Used REPLACE to get rid of unwanted characters.</t>
+  </si>
+  <si>
+    <t>DECISION_TIME</t>
+  </si>
+  <si>
+    <t>Null values</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>This column is unusable since more than 50% of values are missing.</t>
+  </si>
+  <si>
+    <t>TIMESTAMP</t>
+  </si>
+  <si>
+    <t>Column is coming in integer format. Probaby 1900 format from Excel. Time is also inside this value in decimal format. Would be cleaner to separate these values.</t>
+  </si>
+  <si>
+    <t>Column separated into DATE and TIME.
+DATE: Converted to date format calculating the current day by adding the floor number from the TIMESTAMP column (the number without the decimal part) to the date 1899-12-31, and substracting 1, since There is a known Excel bug which records the year 1900 as a leap year, hence counting the incorrect date 1900-02-29. This date was removed by substracting 1.
+TIME: Since the decimal part is a proportion of the seconds in a day, obtained the time column by first getting how many seconds there where for that time, multipling the module of TIMESTAMP % 1 to get decimal part, by 86,400 (quantity of seconds in a day) and used ROUND to get an integer rounded value to represent the quantity of seconds. Then the seconds were converted into time by adding to the time 00:00:00 (12 AM in the morning).</t>
+  </si>
+  <si>
+    <t>AMOUNT</t>
+  </si>
+  <si>
+    <t>It is storing both the amount and the currency as text.</t>
+  </si>
+  <si>
+    <t>Column separated into AMOUNT and CURRENCY. Used SPLIT_PART and separeted by space to get both values in 2 columns.</t>
+  </si>
+  <si>
+    <t>ACCOUNT_FEES</t>
+  </si>
+  <si>
+    <t>Account fees are calculated for every transaction, regardless whether it was blocked or not by the ML model. Blocked transactions do not yield interest since they are not settled.</t>
+  </si>
+  <si>
+    <t>Joined with the cleaned table FRAUD_DECISIONS to determine if transactions where blocked or not. If blocked, then return a 0 for that transaction.</t>
+  </si>
+  <si>
+    <t>MERCHANT_CATEGORY</t>
+  </si>
+  <si>
+    <t>The names are lowecase and separated by underscore. Inconsistent naming for values "web", "web-browser" and "web_payment".</t>
+  </si>
+  <si>
+    <t>Replaced underscores with spaces. Returned Uppercase text. Joined the categories "web", "web-browser" and "web_payment" as just "WEB".</t>
+  </si>
+  <si>
+    <t>Inconsistent values for boolean results. Sometimes return as number, or text in inconsistent way.</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>Replaced "Y" and "TRUE" with 1, since these values represent affirmation. Yes and true.
+Replaced "N" and "FALSE" with 0, since these values represent negation. No and false.</t>
+  </si>
+  <si>
+    <t>INVESTIGATION_COST, CUSTOMER_SUPPORT_COST and LOST_INTERCHANGE</t>
+  </si>
+  <si>
+    <t>These columns are returning negative and positive values. They should all be negative since they are costs. When there is no fraud and the ML model does not catch fraud (TRUE NEGATIVE), the amount should be 0 in all these columns.</t>
+  </si>
+  <si>
+    <t>Joined with the TRANSACTIONS and FRAUD_DECISIONS table and determined that all negative values are from TRUE NEGATIVE results. Returned 0 in all these columns the it is a TRUE POSITIVE, and the other values were changed from positive to negative since they should be represented as debits.</t>
   </si>
 </sst>
 </file>
@@ -349,7 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -381,11 +468,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="30">
+  <dxfs count="60">
     <dxf>
       <font>
         <strike val="0"/>
@@ -571,6 +661,639 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1033,42 +1756,84 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{05C0FE4D-3D83-48C0-8912-23AD1347B2CD}" name="CURRENCY_EXCHANGE_RATES_LOG" displayName="CURRENCY_EXCHANGE_RATES_LOG" ref="A1:E2" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26" totalsRowBorderDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{05C0FE4D-3D83-48C0-8912-23AD1347B2CD}" name="CURRENCY_EXCHANGE_RATES_LOG" displayName="CURRENCY_EXCHANGE_RATES_LOG" ref="A1:E2" totalsRowShown="0" headerRowDxfId="59" dataDxfId="57" headerRowBorderDxfId="58" tableBorderDxfId="56" totalsRowBorderDxfId="55">
   <autoFilter ref="A1:E2" xr:uid="{05C0FE4D-3D83-48C0-8912-23AD1347B2CD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2E40A0B3-AF90-4182-9843-2288801456DE}" name="COLUMN" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{F80B9787-EB7F-4E48-848A-5C6AA8F617DA}" name="ISSUE" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{0AB4CDCB-C236-4A3C-A4A4-9D44F21813D8}" name="ROW_COUNT" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{54E6A82B-991C-4065-96DF-727003752F56}" name="SOLVABLE?" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{7862C159-CC1E-4693-A947-D23804304F60}" name="RESOLUTION" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{2E40A0B3-AF90-4182-9843-2288801456DE}" name="COLUMN" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{F80B9787-EB7F-4E48-848A-5C6AA8F617DA}" name="ISSUE" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{0AB4CDCB-C236-4A3C-A4A4-9D44F21813D8}" name="ROW_COUNT" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{54E6A82B-991C-4065-96DF-727003752F56}" name="SOLVABLE?" dataDxfId="51"/>
+    <tableColumn id="5" xr3:uid="{7862C159-CC1E-4693-A947-D23804304F60}" name="RESOLUTION" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2559DFCC-38D7-4B21-B9B4-4C2119AFCC1B}" name="ACCOUNTS_LOG" displayName="ACCOUNTS_LOG" ref="A1:E9" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16" totalsRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2559DFCC-38D7-4B21-B9B4-4C2119AFCC1B}" name="ACCOUNTS_LOG" displayName="ACCOUNTS_LOG" ref="A1:E9" totalsRowShown="0" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48" tableBorderDxfId="46" totalsRowBorderDxfId="45">
   <autoFilter ref="A1:E9" xr:uid="{2559DFCC-38D7-4B21-B9B4-4C2119AFCC1B}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{24C76CF5-60AC-4D99-B257-103FA77CA877}" name="COLUMN" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{3337A670-71E0-4223-B5A5-44BCF535FADF}" name="ISSUE" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{75E5D8EA-C827-466C-A54E-C6D233FF37A9}" name="ROW_COUNT" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{E754BFA5-49D4-4DE6-974C-68E66960C0FB}" name="SOLVABLE?" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{E655503B-E1BA-4C6B-855C-199DC3D0C0C1}" name="RESOLUTION" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{24C76CF5-60AC-4D99-B257-103FA77CA877}" name="COLUMN" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{3337A670-71E0-4223-B5A5-44BCF535FADF}" name="ISSUE" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{75E5D8EA-C827-466C-A54E-C6D233FF37A9}" name="ROW_COUNT" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{E754BFA5-49D4-4DE6-974C-68E66960C0FB}" name="SOLVABLE?" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{E655503B-E1BA-4C6B-855C-199DC3D0C0C1}" name="RESOLUTION" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80E774B3-ED81-44B3-B55B-CB30FBB2CC6A}" name="CUSTOMERS_LOG" displayName="CUSTOMERS_LOG" ref="A1:E7" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80E774B3-ED81-44B3-B55B-CB30FBB2CC6A}" name="CUSTOMERS_LOG" displayName="CUSTOMERS_LOG" ref="A1:E7" totalsRowShown="0" headerRowDxfId="39" dataDxfId="37" headerRowBorderDxfId="38" tableBorderDxfId="36" totalsRowBorderDxfId="35">
   <autoFilter ref="A1:E7" xr:uid="{80E774B3-ED81-44B3-B55B-CB30FBB2CC6A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{61E96C8D-2220-4567-BB54-92EC049CF4F5}" name="COLUMN" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{D071CD65-CD39-4278-9D0A-DFB78B630E35}" name="ISSUE" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{83A03F84-5429-40D2-9146-4D040C3B0952}" name="ROW_COUNT" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{9E8CE933-1F0D-4B77-B634-8E01CE3B889D}" name="SOLVABLE?" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{FA4FB0EF-2A46-4B38-9DA8-CA7E9F384D25}" name="RESOLUTION" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{61E96C8D-2220-4567-BB54-92EC049CF4F5}" name="COLUMN" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{D071CD65-CD39-4278-9D0A-DFB78B630E35}" name="ISSUE" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{83A03F84-5429-40D2-9146-4D040C3B0952}" name="ROW_COUNT" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{9E8CE933-1F0D-4B77-B634-8E01CE3B889D}" name="SOLVABLE?" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{FA4FB0EF-2A46-4B38-9DA8-CA7E9F384D25}" name="RESOLUTION" dataDxfId="30"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{DFF76B32-0D88-4103-915F-6B62B1B4AFFF}" name="FRAUD_DECISIONS_LOG" displayName="FRAUD_DECISIONS_LOG" ref="A1:E4" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28" headerRowBorderDxfId="26" tableBorderDxfId="27" totalsRowBorderDxfId="25">
+  <autoFilter ref="A1:E4" xr:uid="{DFF76B32-0D88-4103-915F-6B62B1B4AFFF}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{58E14777-AB82-43DC-89AC-E9CEDBDD51C2}" name="COLUMN" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{CD5DC19E-3845-4329-AEBC-C3A33F3DCEB3}" name="ISSUE" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{7C347363-31AE-4A2F-B324-B50D6900D2C2}" name="ROW_COUNT" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{C5B0C625-5DA5-4F0F-B3EA-75D8A4417CC9}" name="SOLVABLE?" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{29A5587B-A438-4F7D-9060-D89A0DC9DBA9}" name="RESOLUTION" dataDxfId="20"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9AFE3C75-C06E-4CDD-9EC4-5D3937D01F5A}" name="TRANSACTIONS_LOG" displayName="TRANSACTIONS_LOG" ref="A1:E6" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" headerRowBorderDxfId="16" tableBorderDxfId="17" totalsRowBorderDxfId="15">
+  <autoFilter ref="A1:E6" xr:uid="{9AFE3C75-C06E-4CDD-9EC4-5D3937D01F5A}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{1F611AEE-665A-48CE-A0D0-B23C83D04AEB}" name="COLUMN" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{B281A476-9E4C-4D0C-9A1C-03B774227A46}" name="ISSUE" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{6759004E-A61B-4380-9379-9C271874DBA3}" name="ROW_COUNT" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{47FCE10C-909B-40AA-9C22-CB2B59DB8A2D}" name="SOLVABLE?" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{F197FA95-C4C9-4E19-9D71-6B25B6A40731}" name="RESOLUTION" dataDxfId="10"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6D850D2E-A420-46EC-963D-C048357A38A4}" name="FRAUD_COSTS_LOG" displayName="FRAUD_COSTS_LOG" ref="A1:E2" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7" totalsRowBorderDxfId="5">
+  <autoFilter ref="A1:E2" xr:uid="{6D850D2E-A420-46EC-963D-C048357A38A4}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{7EC1EFB9-4D04-4CCC-852C-98A4C4AAF1E1}" name="COLUMN" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{346ABBF4-9F6E-4173-8596-D73DD5C40A0C}" name="ISSUE" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{748912C1-766A-4D0E-AEF4-9851D3B5F711}" name="ROW_COUNT" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{03A6C765-E8DC-49D4-9C83-40DC97B0EB10}" name="SOLVABLE?" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{E2841513-C325-4793-9E02-2AAE68390DA4}" name="RESOLUTION" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1754,4 +2519,268 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{583C1207-263E-441F-96F3-023CC51611A0}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="62.7109375" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="89.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="63" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="7">
+        <v>26395</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AB2C2A0-E7B9-4447-A586-29DF92C5451C}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="66.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="103.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="294" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="42" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="84" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="7">
+        <v>2325</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="63" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57A8AFBC-4185-47DE-95E6-051A8A308265}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="43.42578125" customWidth="1"/>
+    <col min="2" max="2" width="60.5703125" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="76" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="126" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="7">
+        <v>47424</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>